<commit_message>
feat(benchmark): write dataset statistics and model comparison sheets to Excel
</commit_message>
<xml_diff>
--- a/docs/Tap_Du_Lieu_Huan_Luyen_Chuan_12Truong.xlsx
+++ b/docs/Tap_Du_Lieu_Huan_Luyen_Chuan_12Truong.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DuLieuHuanLuyen_240Mau" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ThongKe_TapDuLieu" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SoSanh_SVM_vs_PhoBERT" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +37,23 @@
       <name val="Times New Roman"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -49,8 +66,20 @@
         <bgColor rgb="001E3A5F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8EEF5"/>
+        <bgColor rgb="00E8EEF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F4EA"/>
+        <bgColor rgb="00E6F4EA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -72,11 +101,25 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -87,6 +130,36 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -13710,4 +13783,814 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>BẢNG 1: THỐNG KÊ BỘ DỮ LIỆU HUẤN LUYỆN &amp; KIỂM THỬ CHUẨN 12 TRƯỜNG (240 MẪU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Mã lĩnh vực</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Tên lĩnh vực đăng ký (Nhãn)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Tổng mẫu</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Tập Train (75%)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Tập Test (25%)</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Bài báo KH</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Đề tài NCKH</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Mẫu Liên ngành</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>LV-CNTT</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Công nghệ thông tin và Truyền thông</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>LV-DDT</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Kỹ thuật Điện - Điện tử và Tự động hóa</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>LV-CKD</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Kỹ thuật Cơ khí, Chế tạo máy và Giao thông</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>LV-KTQL</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Kinh tế, Quản trị kinh doanh và Tài chính</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>LV-HSMT</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Hóa học, Sinh học, Y Dược và Môi trường</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>LV-XHNV</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Khoa học Xã hội, Nhân văn và Giáo dục học</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Toàn bộ 6 lĩnh vực chuyên ngành (12 trường chuẩn)</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>240</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>180</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>174</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>96</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>BẢNG 2: SO SÁNH TỔNG HỢP TF-IDF + SVM VÀ FINE-TUNING PHOBERT TRÊN TẬP KIỂM THỬ (60 MẪU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Chỉ số đánh giá (Metric)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Mô hình 1: TF-IDF + SVM (LinearSVC)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Mô hình 2: Fine-tuning PhoBERT</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Chênh lệch (PhoBERT vs SVM)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Mô hình tối ưu được chọn</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Precision (Độ xác thực Macro)</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>89.28%</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>95.71%</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>+6.43%</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Fine-tuning PhoBERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Recall (Độ bao phủ Macro)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>88.33%</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>95.0%</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>+6.67%</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Fine-tuning PhoBERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>F1-score (Trung bình điều hòa Macro)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>88.44%</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>94.96%</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>+6.52%</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Fine-tuning PhoBERT (Tối ưu nhất)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Accuracy (Độ chính xác toàn cục)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>88.33%</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>95.0%</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>+6.67%</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Fine-tuning PhoBERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Thời gian suy luận trung bình / 1 hồ sơ</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>2.04 ms</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>37.94 ms</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>+35.9 ms</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Đều đạt thời gian thực (&lt; 50 ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>QUYẾT ĐỊNH LỰA CHỌN CỦA ĐỒ ÁN</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Mô hình Đối chứng (Baseline)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>MÔ HÌNH CHÍNH (PRIMARY MODEL)</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Vượt trội +6.52% F1</t>
+        </is>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Mô hình Học sâu: Tinh chỉnh PhoBERT Tiếng Việt</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>BẢNG 3: SO SÁNH CHI TIẾT PRECISION, RECALL, F1-SCORE THEO TỪNG LĨNH VỰC CHUYÊN NGÀNH</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mã lĩnh vực</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Tên lĩnh vực đăng ký</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>SVM Precision (%)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>SVM Recall (%)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>SVM F1-score (%)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>PhoBERT Precision (%)</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>PhoBERT Recall (%)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>PhoBERT F1-score (%)</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Chênh lệch F1 (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>LV-CNTT</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Công nghệ thông tin và Truyền thông</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>88.89</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>84.20999999999999</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>88.89</v>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>+4.68</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>LV-DDT</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Kỹ thuật Điện - Điện tử và Tự động hóa</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>80</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>88.89</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>94.73999999999999</v>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>+5.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>LV-CKD</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Kỹ thuật Cơ khí, Chế tạo máy và Giao thông</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>+0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>LV-KTQL</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Kinh tế, Quản trị kinh doanh và Tài chính</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>+10.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>LV-HSMT</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Hóa học, Sinh học, Y Dược và Môi trường</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>81.81999999999999</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>85.70999999999999</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>90.91</v>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>+5.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>LV-XHNV</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Khoa học Xã hội, Nhân văn và Giáo dục học</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>81.81999999999999</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>90.91</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>95.23999999999999</v>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>+13.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>LÝ DO LỰA CHỌN FINE-TUNING PHOBERT LÀM MÔ HÌNH CHÍNH CỦA DỰ ÁN:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Lý do 1: Độ chính xác F1-score vượt trội trên cùng tập kiểm thử độc lập: Fine-tuning PhoBERT đạt Macro F1-score 94.96% (Precision 95.71%, Recall 95.0%), cao hơn +6.52% so với TF-IDF + SVM (88.44%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Lý do 2: Giải quyết triệt để bài toán hồ sơ KH&amp;CN liên ngành (Interdisciplinary Records): Mô hình túi từ TF-IDF + SVM chỉ đếm tần suất từ độc lập nên bị nhiễu khi gặp công trình giao thoa (ví dụ: ứng dụng trí tuệ nhân tạo trong tài chính ngân hàng hoặc nghiên cứu ngôn ngữ học thuật ngữ cơ khí - điện tử), trong khi cơ chế Self-Attention hai chiều của PhoBERT nắm bắt chính xác ngữ cảnh chủ đạo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Lý do 3: Hiểu sâu cấu trúc từ ghép và ngữ nghĩa học thuật tiếng Việt: PhoBERT được tiền huấn luyện trên 20GB ngữ liệu tiếng Việt kết hợp tách từ PyVi và mã hóa BPE, giúp nhận diện chính xác các cụm thuật ngữ chuyên ngành phức tạp trong cả 12 trường đầu vào.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Lý do 4: Phân bố xác suất đầu ra (Softmax Confidence) đáng tin cậy hơn cho quy trình thẩm định 5 bước: Xác suất độ tin cậy của PhoBERT phản ánh sát thực tế mức độ chắc chắn ngữ nghĩa, phục vụ trực tiếp cho việc tính Điểm rủi ro lệch nhãn ở Chức năng 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Lý do 5: Thời gian suy luận đáp ứng hoàn hảo yêu cầu thời gian thực: Nhờ đóng băng 8 tầng Transformer bên dưới (Layers 0..7), thời gian phản hồi trung bình của PhoBERT chỉ khoảng 37.94 ms/hồ sơ (nhỏ hơn ngưỡng yêu cầu 50 ms), hoàn toàn phù hợp để làm Mô hình chính thức duy nhất của dự án.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>